<commit_message>
docs: corregir correspondencia de citas legales (art.54, art.132) y normalizar encabezado de criterios de aceptación
</commit_message>
<xml_diff>
--- a/docs/matriz_DEFINITIVA.xlsx
+++ b/docs/matriz_DEFINITIVA.xlsx
@@ -844,7 +844,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="60" customHeight="1" s="48">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -9713,7 +9712,6 @@
     <row r="2" ht="49.5" customHeight="1" s="48">
       <c r="A2" s="54" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="48">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10408,16 +10406,13 @@
       </c>
     </row>
     <row r="53" ht="139.5" customHeight="1" s="48">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="A53" s="66" t="inlineStr">
         <is>
           <t>Reforma LOPSRM 14-11-2025</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>DOF 14-11-2025 (última reforma vigente)</t>
-        </is>
-      </c>
+      <c r="B53" s="58" t="n"/>
+      <c r="C53" s="59" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="66" t="n"/>
@@ -10436,8 +10431,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
@@ -11409,7 +11402,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>1) Apertura del periodo conforme al plazo del contrato y al art. 132 RLOPSRM (estructura de la carátula).
+          <t>1) Apertura del periodo conforme al plazo del contrato y al art. 132 RLOPSRM (documentos soporte que acompañan la estimación).
 2) Cálculos administrativos en la carátula: anticipo y su amortización (art. 50 LOPSRM), retenciones legales (5 al millar conforme al art. 191 LFD) y deductivas por penalizaciones (art. 46 Bis LOPSRM).</t>
         </is>
       </c>
@@ -11605,7 +11598,7 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>1) Plazo de revisión: 15 días naturales (supervisión) + 5 días para autorización por residencia, dentro de los 20 días del art. 54 LOPSRM.
+          <t>1) Plazo de revisión y autorización: hasta 15 días naturales tras la presentación de la estimación (art. 54 LOPSRM). El pago corre por separado (ver SRV-07-01).
 2) Afirmativa ficta del art. 133 RLOPSRM: si no se emiten observaciones en el plazo, se considera que no las hay.
 3) Anticipos y amortización conforme art. 50 LOPSRM; retenciones y deductivas según contrato.</t>
         </is>

</xml_diff>

<commit_message>
docs: blindar 7 HU prioritarias (servicios + historias coherentes + correcciones del profe sprint 2/3)
</commit_message>
<xml_diff>
--- a/docs/matriz_DEFINITIVA.xlsx
+++ b/docs/matriz_DEFINITIVA.xlsx
@@ -10719,20 +10719,25 @@
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
-          <t>• Captura los datos generales del contrato y el PDF firmado.
-• Carga el catálogo de conceptos completo con clave, descripción, unidad, precio y cantidad.
-• Registra el programa de obra mes a mes por concepto.
-• Guarda los elementos jurídicos del contratista.
-• Versiona la configuración inicial para que después pueda actualizarse por modificatorios.</t>
+          <t>• Captura los datos generales del contrato (folio único, partes, monto, plazos, modalidad de pago).
+• Carga el catálogo de conceptos completo (clave, descripción, unidad, precio unitario, cantidad contratada).
+• Registra el programa de obra (calendario de ejecución por concepto, mes a mes).
+• Registra los elementos jurídicos, separando los de la dependencia (representante, facultades, fundamento de contratación) de los del contratista (representante legal, datos fiscales, poder).
+• Registra las garantías: póliza de anticipo, póliza de cumplimiento y garantía de vicios ocultos según lo pactado (cláusula y/o póliza) — fundamento art. 48 LOPSRM.
+• Registra el plan de amortización del anticipo y las penalizaciones aplicables, incluida la retención del 5 al millar sobre estimaciones (art. 191 LFD).
+• Guarda el PDF firmado del contrato como respaldo documental.
+• Valida que los campos obligatorios estén completos y el folio sea único antes de guardar.
+• Versiona la configuración inicial para que pueda actualizarse por modificatorios (SRV-01-03).</t>
         </is>
       </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
-          <t>• No genera el contrato (asume que ya está firmado fuera del sistema).
-• No edita el PDF del contrato firmado (es inmutable).
-• No valida si el contrato cumple legalmente (eso ya lo hizo la dependencia antes de firmarlo).
-• No interactúa con CompraNet, SAT ni sistemas externos.
-• No autoriza ni rechaza el contrato (solo lo captura).</t>
+          <t>• No genera el contrato (ya está firmado fuera del sistema antes de capturarse).
+• No edita el PDF firmado (es inmutable; cualquier cambio requiere modificatorio).
+• No valida la legalidad del contrato (lo hizo la dependencia antes de firmar).
+• No interactúa con CompraNet, SAT ni afianzadoras.
+• No autoriza ni rechaza el contrato (solo captura).
+• No registra estimaciones ni pagos (SRV-04-* / SRV-07-*).</t>
         </is>
       </c>
       <c r="G2" s="15" t="n"/>
@@ -10966,18 +10971,19 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>• Grafica la curva S del contrato (programado vs ejecutado vs financiero).
-• Muestra el cruce concepto × periodo (mes por mes).
-• Filtra por concepto, periodo o estado de ejecución.
-• Calcula el porcentaje de avance global y por concepto.</t>
+          <t>• Visualiza el programa de obra como matriz concepto × periodo (tipo Gantt), marcando con color los periodos ejecutados vs no ejecutados respecto a lo programado.
+• Muestra el catálogo de conceptos del contrato (lista consultable).
+• Grafica las curvas de avance: programado vs ejecutado vs financiero (curva S).
+• Filtra por concepto, periodo o estado de ejecución; calcula el porcentaje de avance global y por concepto.</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>• No registra el avance (eso lo hace SRV-02-02 y la bitácora).
-• No genera alertas (eso lo hace SRV-02-03, y solo si el usuario las configura).
-• No exporta la gráfica a PDF (eso lo hace SRV-06-03).
-• No proyecta cuándo terminará el contrato (es visualización del estado actual, no predicción).</t>
+          <t>• No registra el avance (SRV-02-02 y la bitácora).
+• No edita el catálogo ni el programa (el alta es de SRV-01-01).
+• No genera alertas (SRV-02-03).
+• No exporta a PDF (SRV-06-03).
+• No proyecta la fecha de término (muestra estado actual, no predicción).</t>
         </is>
       </c>
       <c r="G6" s="15" t="n"/>
@@ -11141,18 +11147,20 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>• Genera la bitácora electrónica única para el contrato.
-• Liga al contratista, la supervisión y la residencia con sus datos de contacto.
-• Define quiénes están autorizados a firmar por cada parte.
-• Marca la fecha y hora de apertura como evento formal.
-• Habilita el módulo de bitácora para emitir notas (SRV-03-02).</t>
+          <t>• Apertura la bitácora electrónica única del contrato en la fecha de entrega del sitio de los trabajos, evento que marca el inicio formal y legal de la comunicación vinculante entre las partes (art. 122 RLOPSRM).
+• Liga a las tres partes (dependencia, supervisión, contratista) con sus datos de contacto y sus representantes autorizados a firmar (residente, supervisor externo si existe, superintendente de construcción).
+• Registra la primera nota (nota de apertura) con los datos obligatorios: identificación del contrato, objeto de los trabajos, datos financieros, cronograma contractual y registro de firmas.
+• Captura la firma conjunta de los tres representantes al aperturar.
+• Marca la fecha y hora de apertura como evento formal inalterable.
+• Habilita el módulo de notas (SRV-03-02).</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>• No emite notas (eso lo hace SRV-03-02).
-• No se puede repetir: una vez abierta, no se vuelve a abrir.
-• No cierra la bitácora (el cierre es parte del finiquito, Etapa 2).</t>
+          <t>• No emite notas posteriores a la apertura (SRV-03-02).
+• No se vuelve a aperturar una vez registrada la apertura.
+• No cierra la bitácora (es parte del finiquito, Etapa 2 — fuera de alcance).
+• No registra apertura sin la firma conjunta de los tres autorizados.</t>
         </is>
       </c>
       <c r="G9" s="15" t="n"/>
@@ -11200,20 +11208,22 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>• Permite emitir las notas tipificadas que corresponden al rol del usuario.
-• Asigna folio correlativo automático, fecha y hora del sistema y firmante.
-• Permite vincular respuestas a una nota previa por referencia explícita.
+          <t>• Permite emitir las notas tipificadas que corresponden al rol del usuario, pudiendo incorporar también otro tipo de nota para registrar eventos no tipificados.
+• Asigna folio correlativo automático (sin saltos, manejando concurrencia de los tres usuarios), fecha y hora del sistema y firmante.
 • Acepta los eventos formales del contrato: causas de atraso, instrucciones técnicas, entregas de obra, acuerdos entre partes, solicitudes de información y respuestas.
+• Permite vincular respuestas o correcciones a una nota previa por referencia explícita (formato «dice / debe decir» para correcciones).
+• Captura la firma conjunta de los tres participantes (residente, supervisión y contratista) en cada nota emitida — comportamiento de libro de actas.
 • Permite adjuntar archivos como soporte (fotografías, planos, oficios) hasta 10 MB por archivo.
-• Garantiza inmutabilidad: las notas firmadas no se pueden modificar ni eliminar.</t>
+• Garantiza inmutabilidad: una vez firmada, la nota no se puede modificar ni eliminar (correcciones = nota vinculada nueva).
+• Fundamento: arts. 122 y 125 RLOPSRM.</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
           <t>• No permite borrar notas (las correcciones se hacen con notas nuevas vinculadas).
-• No permite a un rol emitir notas que no le corresponden (residente no puede emitir nota de contratista).
+• No permite a un rol emitir notas tipificadas que no le corresponden (residente no puede emitir una nota propia del contratista).
 • No valida el contenido técnico de la nota (la responsabilidad sigue siendo de quien firma).
-• No envía las notas a entidades externas (es bitácora interna del contrato).</t>
+• No envía las notas a entidades externas (bitácora interna del contrato).</t>
         </is>
       </c>
       <c r="G10" s="15" t="inlineStr">
@@ -11267,17 +11277,18 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>• Buscador con filtros: tipo, fecha, firmante, estatus, tema.
+          <t>• Buscador de notas de la bitácora con los siguientes filtros combinables con lógica Y (AND): tipo de nota, rango de fechas (desde / hasta), firmante (quién escribió la nota), vínculo (notas vinculadas a otra previa / sin vínculo), palabra clave sobre el contenido (búsqueda simple por coincidencia de texto, mediante PostgreSQL ILIKE).
 • Filtra por rol del emisor o destinatario.
-• Permite seleccionar varias notas para adjuntar a una estimación.
-• Exportación básica del listado (PDF/Excel).</t>
+• Permite seleccionar varias notas del resultado y exportarlas a formato Excel.
+• Devuelve solo las notas que cumplen simultáneamente todos los filtros aplicados.</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
           <t>• No edita las notas encontradas.
 • No re-firma las notas (la firma sigue siendo la original).
-• No hace búsqueda semántica avanzada (es búsqueda por metadatos, no por contenido completo).</t>
+• No hace búsqueda semántica (es coincidencia simple de texto, no análisis semántico).
+• No adjunta notas a una estimación (esa función se realiza desde el armado de la estimación, SRV-04-01).</t>
         </is>
       </c>
       <c r="G11" s="15" t="n"/>
@@ -11385,16 +11396,16 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>• Abre el periodo de estimación N dentro del plazo legal (art. 54 LOPSRM).
-• Permite armar carátula, números generadores, registro fotográfico y soportes.
-• Liga las notas de bitácora del periodo a la estimación.
+          <t>• Abre el periodo de estimación N dentro del plazo legal de presentación (art. 54 LOPSRM).
+• Permite armar la carátula, los números generadores, el registro fotográfico y los soportes de la estimación.
+• Permite buscar y seleccionar notas de bitácora del periodo (usando SRV-03-03) para vincularlas a la estimación.
 • Guarda toda la estimación como una sola entidad cohesionada.
-• Calcula automáticamente totales por concepto y periodo.</t>
+• Calcula automáticamente los totales por concepto y periodo, y las cantidades de la carátula: anticipo amortizado, retenciones legales (5 al millar, art. 191 LFD) y deductivas por penalizaciones según el contrato.</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>• No envía la estimación a revisión (eso es SRV-04-02).
+          <t>• No envía la estimación a revisión (SRV-04-02).
 • No valida internamente contra catálogo o programa (eso lo hace la supervisión en SRV-05-01).
 • No carga conceptos que no estén en el catálogo del contrato.
 • No permite mezclar periodos (una estimación es de un solo periodo).</t>
@@ -11971,17 +11982,19 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>• Permite a Finanzas capturar el pago efectuado.
-• Registra fecha, importe, referencia bancaria y observaciones.
+          <t>• Permite a Finanzas registrar el pago ya realizado de una estimación autorizada.
+• Captura los datos obligatorios: fecha, importe, referencia bancaria, observaciones y usuario que realizó el registro.
+• Valida que todos los datos obligatorios estén completos antes de permitir guardar el registro.
 • Actualiza el avance financiero del contrato.
-• Cierra el ciclo de la estimación pagada.</t>
+• Marca la estimación como pagada y cierra el ciclo de esa estimación.</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>• No transfiere el dinero (esa transferencia es operación bancaria fuera del sistema).
-• No emite el comprobante de pago.
-• No registra pagos parciales (el pago se asume completo según lo autorizado).</t>
+          <t>• No transfiere el dinero (esa operación es bancaria, fuera del sistema).
+• No emite el comprobante de pago (lo emite el banco).
+• No registra pagos parciales (el pago se asume completo según lo autorizado).
+• No genera la instrucción de pago (eso lo hace SRV-07-01, HU-20).</t>
         </is>
       </c>
       <c r="G22" s="15" t="n"/>

</xml_diff>